<commit_message>
Commit: las salidas estan lista. leer  los archivos de simulacion_ingreso y salidas.
</commit_message>
<xml_diff>
--- a/movimientos.xlsx
+++ b/movimientos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1699" uniqueCount="452">
   <si>
     <t>Nº de Procesado</t>
   </si>
@@ -1055,6 +1055,321 @@
   </si>
   <si>
     <t>12:25:01</t>
+  </si>
+  <si>
+    <t>2314977</t>
+  </si>
+  <si>
+    <t>260001921</t>
+  </si>
+  <si>
+    <t>16:16:50</t>
+  </si>
+  <si>
+    <t>2314978</t>
+  </si>
+  <si>
+    <t>260001922</t>
+  </si>
+  <si>
+    <t>16:19:08</t>
+  </si>
+  <si>
+    <t>2314979</t>
+  </si>
+  <si>
+    <t>260001923</t>
+  </si>
+  <si>
+    <t>16:20:56</t>
+  </si>
+  <si>
+    <t>2314980</t>
+  </si>
+  <si>
+    <t>260001924</t>
+  </si>
+  <si>
+    <t>16:22:39</t>
+  </si>
+  <si>
+    <t>2314981</t>
+  </si>
+  <si>
+    <t>260001925</t>
+  </si>
+  <si>
+    <t>16:24:22</t>
+  </si>
+  <si>
+    <t>5392775</t>
+  </si>
+  <si>
+    <t>260041853</t>
+  </si>
+  <si>
+    <t>16:37:48</t>
+  </si>
+  <si>
+    <t>06732F05</t>
+  </si>
+  <si>
+    <t>06732F0201</t>
+  </si>
+  <si>
+    <t>5392776</t>
+  </si>
+  <si>
+    <t>260041854</t>
+  </si>
+  <si>
+    <t>16:38:56</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>06732F03</t>
+  </si>
+  <si>
+    <t>06732F0301</t>
+  </si>
+  <si>
+    <t>5392777</t>
+  </si>
+  <si>
+    <t>16:39:57</t>
+  </si>
+  <si>
+    <t>06732F04</t>
+  </si>
+  <si>
+    <t>06732F0401</t>
+  </si>
+  <si>
+    <t>5392778</t>
+  </si>
+  <si>
+    <t>16:41:01</t>
+  </si>
+  <si>
+    <t>06732F0501</t>
+  </si>
+  <si>
+    <t>5392779</t>
+  </si>
+  <si>
+    <t>260041855</t>
+  </si>
+  <si>
+    <t>16:42:18</t>
+  </si>
+  <si>
+    <t>5392780</t>
+  </si>
+  <si>
+    <t>260041856</t>
+  </si>
+  <si>
+    <t>16:47:41</t>
+  </si>
+  <si>
+    <t>5392781</t>
+  </si>
+  <si>
+    <t>16:49:09</t>
+  </si>
+  <si>
+    <t>SISMED: Por favor tiene que elegir el Concepto</t>
+  </si>
+  <si>
+    <t>5392782</t>
+  </si>
+  <si>
+    <t>16:50:33</t>
+  </si>
+  <si>
+    <t>8455087</t>
+  </si>
+  <si>
+    <t>260001931</t>
+  </si>
+  <si>
+    <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>19:22:05</t>
+  </si>
+  <si>
+    <t>8455088</t>
+  </si>
+  <si>
+    <t>19:23:59</t>
+  </si>
+  <si>
+    <t>SISMED: Debe existir el Almacen Virtual Destino</t>
+  </si>
+  <si>
+    <t>8455089</t>
+  </si>
+  <si>
+    <t>19:25:57</t>
+  </si>
+  <si>
+    <t>8455090</t>
+  </si>
+  <si>
+    <t>19:28:00</t>
+  </si>
+  <si>
+    <t>8455091</t>
+  </si>
+  <si>
+    <t>19:30:48</t>
+  </si>
+  <si>
+    <t>1808129</t>
+  </si>
+  <si>
+    <t>260001932</t>
+  </si>
+  <si>
+    <t>19:55:56</t>
+  </si>
+  <si>
+    <t>5646242</t>
+  </si>
+  <si>
+    <t>260041857</t>
+  </si>
+  <si>
+    <t>21:28:49</t>
+  </si>
+  <si>
+    <t>5646243</t>
+  </si>
+  <si>
+    <t>260041858</t>
+  </si>
+  <si>
+    <t>21:30:08</t>
+  </si>
+  <si>
+    <t>5646244</t>
+  </si>
+  <si>
+    <t>260041859</t>
+  </si>
+  <si>
+    <t>21:31:50</t>
+  </si>
+  <si>
+    <t>4903025</t>
+  </si>
+  <si>
+    <t>260041862</t>
+  </si>
+  <si>
+    <t>22:18:27</t>
+  </si>
+  <si>
+    <t>4903026</t>
+  </si>
+  <si>
+    <t>260041863</t>
+  </si>
+  <si>
+    <t>22:19:56</t>
+  </si>
+  <si>
+    <t>4903027</t>
+  </si>
+  <si>
+    <t>260041864</t>
+  </si>
+  <si>
+    <t>22:21:20</t>
+  </si>
+  <si>
+    <t>4903028</t>
+  </si>
+  <si>
+    <t>260041865</t>
+  </si>
+  <si>
+    <t>22:22:52</t>
+  </si>
+  <si>
+    <t>8054400</t>
+  </si>
+  <si>
+    <t>260041866</t>
+  </si>
+  <si>
+    <t>22:27:09</t>
+  </si>
+  <si>
+    <t>8054401</t>
+  </si>
+  <si>
+    <t>260041867</t>
+  </si>
+  <si>
+    <t>22:28:32</t>
+  </si>
+  <si>
+    <t>8054402</t>
+  </si>
+  <si>
+    <t>260041868</t>
+  </si>
+  <si>
+    <t>22:29:56</t>
+  </si>
+  <si>
+    <t>8054403</t>
+  </si>
+  <si>
+    <t>260041869</t>
+  </si>
+  <si>
+    <t>22:31:19</t>
+  </si>
+  <si>
+    <t>8054404</t>
+  </si>
+  <si>
+    <t>260041870</t>
+  </si>
+  <si>
+    <t>22:32:43</t>
+  </si>
+  <si>
+    <t>8054405</t>
+  </si>
+  <si>
+    <t>260041871</t>
+  </si>
+  <si>
+    <t>22:38:13</t>
+  </si>
+  <si>
+    <t>8054406</t>
+  </si>
+  <si>
+    <t>260041872</t>
+  </si>
+  <si>
+    <t>22:39:45</t>
+  </si>
+  <si>
+    <t>8054407</t>
+  </si>
+  <si>
+    <t>260041873</t>
+  </si>
+  <si>
+    <t>22:41:26</t>
   </si>
 </sst>
 </file>
@@ -1116,8 +1431,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:Y110" totalsRowShown="0">
-  <autoFilter ref="A1:Y110"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:Y144" totalsRowShown="0">
+  <autoFilter ref="A1:Y144"/>
   <tableColumns count="25">
     <tableColumn id="1" name="Nº de Procesado" dataDxfId="0"/>
     <tableColumn id="2" name="Nº correlativo Ksalud" dataDxfId="1"/>
@@ -1434,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y110"/>
+  <dimension ref="A1:Y144"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:25">
@@ -7513,6 +7828,1788 @@
       </c>
       <c r="Y110" s="2"/>
     </row>
+    <row r="111" spans="1:25">
+      <c r="A111" s="1">
+        <v>101</v>
+      </c>
+      <c r="B111" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E111" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G111" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H111" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I111" s="2"/>
+      <c r="J111" s="2"/>
+      <c r="K111" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L111" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M111" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N111" s="2"/>
+      <c r="O111" s="2"/>
+      <c r="P111" s="2"/>
+      <c r="Q111" s="2"/>
+      <c r="R111" s="2"/>
+      <c r="S111" s="2"/>
+      <c r="T111" s="2"/>
+      <c r="U111" s="2"/>
+      <c r="V111" s="2"/>
+      <c r="W111" s="2"/>
+      <c r="X111" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y111" s="2"/>
+    </row>
+    <row r="112" spans="1:25">
+      <c r="A112" s="1">
+        <v>102</v>
+      </c>
+      <c r="B112" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E112" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G112" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H112" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I112" s="2"/>
+      <c r="J112" s="2"/>
+      <c r="K112" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L112" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M112" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N112" s="2"/>
+      <c r="O112" s="2"/>
+      <c r="P112" s="2"/>
+      <c r="Q112" s="2"/>
+      <c r="R112" s="2"/>
+      <c r="S112" s="2"/>
+      <c r="T112" s="2"/>
+      <c r="U112" s="2"/>
+      <c r="V112" s="2"/>
+      <c r="W112" s="2"/>
+      <c r="X112" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y112" s="2"/>
+    </row>
+    <row r="113" spans="1:25">
+      <c r="A113" s="1">
+        <v>103</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="C113" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G113" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H113" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I113" s="2"/>
+      <c r="J113" s="2"/>
+      <c r="K113" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L113" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M113" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N113" s="2"/>
+      <c r="O113" s="2"/>
+      <c r="P113" s="2"/>
+      <c r="Q113" s="2"/>
+      <c r="R113" s="2"/>
+      <c r="S113" s="2"/>
+      <c r="T113" s="2"/>
+      <c r="U113" s="2"/>
+      <c r="V113" s="2"/>
+      <c r="W113" s="2"/>
+      <c r="X113" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y113" s="2"/>
+    </row>
+    <row r="114" spans="1:25">
+      <c r="A114" s="1">
+        <v>104</v>
+      </c>
+      <c r="B114" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C114" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I114" s="2"/>
+      <c r="J114" s="2"/>
+      <c r="K114" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L114" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M114" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N114" s="2"/>
+      <c r="O114" s="2"/>
+      <c r="P114" s="2"/>
+      <c r="Q114" s="2"/>
+      <c r="R114" s="2"/>
+      <c r="S114" s="2"/>
+      <c r="T114" s="2"/>
+      <c r="U114" s="2"/>
+      <c r="V114" s="2"/>
+      <c r="W114" s="2"/>
+      <c r="X114" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y114" s="2"/>
+    </row>
+    <row r="115" spans="1:25">
+      <c r="A115" s="1">
+        <v>105</v>
+      </c>
+      <c r="B115" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G115" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H115" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I115" s="2"/>
+      <c r="J115" s="2"/>
+      <c r="K115" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L115" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M115" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N115" s="2"/>
+      <c r="O115" s="2"/>
+      <c r="P115" s="2"/>
+      <c r="Q115" s="2"/>
+      <c r="R115" s="2"/>
+      <c r="S115" s="2"/>
+      <c r="T115" s="2"/>
+      <c r="U115" s="2"/>
+      <c r="V115" s="2"/>
+      <c r="W115" s="2"/>
+      <c r="X115" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y115" s="2"/>
+    </row>
+    <row r="116" spans="1:25">
+      <c r="A116" s="1">
+        <v>106</v>
+      </c>
+      <c r="B116" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="C116" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G116" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H116" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I116" s="2"/>
+      <c r="J116" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K116" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L116" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="M116" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N116" s="2"/>
+      <c r="O116" s="2"/>
+      <c r="P116" s="2"/>
+      <c r="Q116" s="2"/>
+      <c r="R116" s="2"/>
+      <c r="S116" s="2"/>
+      <c r="T116" s="2"/>
+      <c r="U116" s="2"/>
+      <c r="V116" s="2"/>
+      <c r="W116" s="2"/>
+      <c r="X116" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y116" s="2"/>
+    </row>
+    <row r="117" spans="1:25">
+      <c r="A117" s="1">
+        <v>107</v>
+      </c>
+      <c r="B117" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="C117" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E117" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G117" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H117" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I117" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="J117" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="K117" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L117" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="M117" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N117" s="2"/>
+      <c r="O117" s="2"/>
+      <c r="P117" s="2"/>
+      <c r="Q117" s="2"/>
+      <c r="R117" s="2"/>
+      <c r="S117" s="2"/>
+      <c r="T117" s="2"/>
+      <c r="U117" s="2"/>
+      <c r="V117" s="2"/>
+      <c r="W117" s="2"/>
+      <c r="X117" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y117" s="2"/>
+    </row>
+    <row r="118" spans="1:25">
+      <c r="A118" s="1">
+        <v>108</v>
+      </c>
+      <c r="B118" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C118" s="2"/>
+      <c r="D118" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G118" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="K118" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L118" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="M118" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N118" s="2"/>
+      <c r="O118" s="2"/>
+      <c r="P118" s="2"/>
+      <c r="Q118" s="2"/>
+      <c r="R118" s="2"/>
+      <c r="S118" s="2"/>
+      <c r="T118" s="2"/>
+      <c r="U118" s="2"/>
+      <c r="V118" s="2"/>
+      <c r="W118" s="2"/>
+      <c r="X118" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y118" s="2"/>
+    </row>
+    <row r="119" spans="1:25">
+      <c r="A119" s="1">
+        <v>109</v>
+      </c>
+      <c r="B119" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="C119" s="2"/>
+      <c r="D119" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H119" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I119" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="K119" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L119" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="M119" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N119" s="2"/>
+      <c r="O119" s="2"/>
+      <c r="P119" s="2"/>
+      <c r="Q119" s="2"/>
+      <c r="R119" s="2"/>
+      <c r="S119" s="2"/>
+      <c r="T119" s="2"/>
+      <c r="U119" s="2"/>
+      <c r="V119" s="2"/>
+      <c r="W119" s="2"/>
+      <c r="X119" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y119" s="2"/>
+    </row>
+    <row r="120" spans="1:25">
+      <c r="A120" s="1">
+        <v>110</v>
+      </c>
+      <c r="B120" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="C120" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E120" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G120" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H120" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I120" s="2"/>
+      <c r="J120" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="K120" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L120" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="M120" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N120" s="2"/>
+      <c r="O120" s="2"/>
+      <c r="P120" s="2"/>
+      <c r="Q120" s="2"/>
+      <c r="R120" s="2"/>
+      <c r="S120" s="2"/>
+      <c r="T120" s="2"/>
+      <c r="U120" s="2"/>
+      <c r="V120" s="2"/>
+      <c r="W120" s="2"/>
+      <c r="X120" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y120" s="2"/>
+    </row>
+    <row r="121" spans="1:25">
+      <c r="A121" s="1">
+        <v>111</v>
+      </c>
+      <c r="B121" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="C121" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E121" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I121" s="2"/>
+      <c r="J121" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K121" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L121" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M121" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N121" s="2"/>
+      <c r="O121" s="2"/>
+      <c r="P121" s="2"/>
+      <c r="Q121" s="2"/>
+      <c r="R121" s="2"/>
+      <c r="S121" s="2"/>
+      <c r="T121" s="2"/>
+      <c r="U121" s="2"/>
+      <c r="V121" s="2"/>
+      <c r="W121" s="2"/>
+      <c r="X121" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y121" s="2"/>
+    </row>
+    <row r="122" spans="1:25">
+      <c r="A122" s="1">
+        <v>112</v>
+      </c>
+      <c r="B122" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="C122" s="2"/>
+      <c r="D122" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E122" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G122" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I122" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="J122" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K122" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L122" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M122" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N122" s="2"/>
+      <c r="O122" s="2"/>
+      <c r="P122" s="2"/>
+      <c r="Q122" s="2"/>
+      <c r="R122" s="2"/>
+      <c r="S122" s="2"/>
+      <c r="T122" s="2"/>
+      <c r="U122" s="2"/>
+      <c r="V122" s="2"/>
+      <c r="W122" s="2"/>
+      <c r="X122" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y122" s="2"/>
+    </row>
+    <row r="123" spans="1:25">
+      <c r="A123" s="1">
+        <v>113</v>
+      </c>
+      <c r="B123" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C123" s="2"/>
+      <c r="D123" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="E123" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I123" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K123" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L123" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M123" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N123" s="2"/>
+      <c r="O123" s="2"/>
+      <c r="P123" s="2"/>
+      <c r="Q123" s="2"/>
+      <c r="R123" s="2"/>
+      <c r="S123" s="2"/>
+      <c r="T123" s="2"/>
+      <c r="U123" s="2"/>
+      <c r="V123" s="2"/>
+      <c r="W123" s="2"/>
+      <c r="X123" s="1">
+        <v>3</v>
+      </c>
+      <c r="Y123" s="2"/>
+    </row>
+    <row r="124" spans="1:25">
+      <c r="A124" s="1">
+        <v>114</v>
+      </c>
+      <c r="B124" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="C124" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I124" s="2"/>
+      <c r="J124" s="2"/>
+      <c r="K124" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L124" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M124" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N124" s="2"/>
+      <c r="O124" s="2"/>
+      <c r="P124" s="2"/>
+      <c r="Q124" s="2"/>
+      <c r="R124" s="2"/>
+      <c r="S124" s="2"/>
+      <c r="T124" s="2"/>
+      <c r="U124" s="2"/>
+      <c r="V124" s="2"/>
+      <c r="W124" s="2"/>
+      <c r="X124" s="1">
+        <v>33</v>
+      </c>
+      <c r="Y124" s="2"/>
+    </row>
+    <row r="125" spans="1:25">
+      <c r="A125" s="1">
+        <v>115</v>
+      </c>
+      <c r="B125" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C125" s="2"/>
+      <c r="D125" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I125" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J125" s="2"/>
+      <c r="K125" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L125" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M125" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N125" s="2"/>
+      <c r="O125" s="2"/>
+      <c r="P125" s="2"/>
+      <c r="Q125" s="2"/>
+      <c r="R125" s="2"/>
+      <c r="S125" s="2"/>
+      <c r="T125" s="2"/>
+      <c r="U125" s="2"/>
+      <c r="V125" s="2"/>
+      <c r="W125" s="2"/>
+      <c r="X125" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y125" s="2"/>
+    </row>
+    <row r="126" spans="1:25">
+      <c r="A126" s="1">
+        <v>116</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="C126" s="2"/>
+      <c r="D126" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I126" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="J126" s="2"/>
+      <c r="K126" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="L126" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M126" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N126" s="2"/>
+      <c r="O126" s="2"/>
+      <c r="P126" s="2"/>
+      <c r="Q126" s="2"/>
+      <c r="R126" s="2"/>
+      <c r="S126" s="2"/>
+      <c r="T126" s="2"/>
+      <c r="U126" s="2"/>
+      <c r="V126" s="2"/>
+      <c r="W126" s="2"/>
+      <c r="X126" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y126" s="2"/>
+    </row>
+    <row r="127" spans="1:25">
+      <c r="A127" s="1">
+        <v>117</v>
+      </c>
+      <c r="B127" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C127" s="2"/>
+      <c r="D127" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E127" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G127" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H127" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I127" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J127" s="2"/>
+      <c r="K127" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L127" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M127" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N127" s="2"/>
+      <c r="O127" s="2"/>
+      <c r="P127" s="2"/>
+      <c r="Q127" s="2"/>
+      <c r="R127" s="2"/>
+      <c r="S127" s="2"/>
+      <c r="T127" s="2"/>
+      <c r="U127" s="2"/>
+      <c r="V127" s="2"/>
+      <c r="W127" s="2"/>
+      <c r="X127" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y127" s="2"/>
+    </row>
+    <row r="128" spans="1:25">
+      <c r="A128" s="1">
+        <v>118</v>
+      </c>
+      <c r="B128" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="C128" s="2"/>
+      <c r="D128" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H128" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I128" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="J128" s="2"/>
+      <c r="K128" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L128" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M128" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N128" s="2"/>
+      <c r="O128" s="2"/>
+      <c r="P128" s="2"/>
+      <c r="Q128" s="2"/>
+      <c r="R128" s="2"/>
+      <c r="S128" s="2"/>
+      <c r="T128" s="2"/>
+      <c r="U128" s="2"/>
+      <c r="V128" s="2"/>
+      <c r="W128" s="2"/>
+      <c r="X128" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y128" s="2"/>
+    </row>
+    <row r="129" spans="1:25">
+      <c r="A129" s="1">
+        <v>119</v>
+      </c>
+      <c r="B129" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E129" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G129" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="H129" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I129" s="2"/>
+      <c r="J129" s="2"/>
+      <c r="K129" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L129" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M129" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N129" s="2"/>
+      <c r="O129" s="2"/>
+      <c r="P129" s="2"/>
+      <c r="Q129" s="2"/>
+      <c r="R129" s="2"/>
+      <c r="S129" s="2"/>
+      <c r="T129" s="2"/>
+      <c r="U129" s="2"/>
+      <c r="V129" s="2"/>
+      <c r="W129" s="2"/>
+      <c r="X129" s="1">
+        <v>4</v>
+      </c>
+      <c r="Y129" s="2"/>
+    </row>
+    <row r="130" spans="1:25">
+      <c r="A130" s="1">
+        <v>120</v>
+      </c>
+      <c r="B130" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C130" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E130" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G130" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H130" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I130" s="2"/>
+      <c r="J130" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K130" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L130" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M130" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N130" s="2"/>
+      <c r="O130" s="2"/>
+      <c r="P130" s="2"/>
+      <c r="Q130" s="2"/>
+      <c r="R130" s="2"/>
+      <c r="S130" s="2"/>
+      <c r="T130" s="2"/>
+      <c r="U130" s="2"/>
+      <c r="V130" s="2"/>
+      <c r="W130" s="2"/>
+      <c r="X130" s="1">
+        <v>33</v>
+      </c>
+      <c r="Y130" s="2"/>
+    </row>
+    <row r="131" spans="1:25">
+      <c r="A131" s="1">
+        <v>121</v>
+      </c>
+      <c r="B131" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E131" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I131" s="2"/>
+      <c r="J131" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K131" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L131" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M131" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N131" s="2"/>
+      <c r="O131" s="2"/>
+      <c r="P131" s="2"/>
+      <c r="Q131" s="2"/>
+      <c r="R131" s="2"/>
+      <c r="S131" s="2"/>
+      <c r="T131" s="2"/>
+      <c r="U131" s="2"/>
+      <c r="V131" s="2"/>
+      <c r="W131" s="2"/>
+      <c r="X131" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y131" s="2"/>
+    </row>
+    <row r="132" spans="1:25">
+      <c r="A132" s="1">
+        <v>122</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="C132" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I132" s="2"/>
+      <c r="J132" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K132" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L132" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M132" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N132" s="2"/>
+      <c r="O132" s="2"/>
+      <c r="P132" s="2"/>
+      <c r="Q132" s="2"/>
+      <c r="R132" s="2"/>
+      <c r="S132" s="2"/>
+      <c r="T132" s="2"/>
+      <c r="U132" s="2"/>
+      <c r="V132" s="2"/>
+      <c r="W132" s="2"/>
+      <c r="X132" s="1">
+        <v>5</v>
+      </c>
+      <c r="Y132" s="2"/>
+    </row>
+    <row r="133" spans="1:25">
+      <c r="A133" s="1">
+        <v>123</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E133" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H133" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I133" s="2"/>
+      <c r="J133" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K133" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L133" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M133" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N133" s="2"/>
+      <c r="O133" s="2"/>
+      <c r="P133" s="2"/>
+      <c r="Q133" s="2"/>
+      <c r="R133" s="2"/>
+      <c r="S133" s="2"/>
+      <c r="T133" s="2"/>
+      <c r="U133" s="2"/>
+      <c r="V133" s="2"/>
+      <c r="W133" s="2"/>
+      <c r="X133" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y133" s="2"/>
+    </row>
+    <row r="134" spans="1:25">
+      <c r="A134" s="1">
+        <v>124</v>
+      </c>
+      <c r="B134" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="C134" s="2" t="s">
+        <v>420</v>
+      </c>
+      <c r="D134" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G134" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H134" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I134" s="2"/>
+      <c r="J134" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K134" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="L134" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M134" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N134" s="2"/>
+      <c r="O134" s="2"/>
+      <c r="P134" s="2"/>
+      <c r="Q134" s="2"/>
+      <c r="R134" s="2"/>
+      <c r="S134" s="2"/>
+      <c r="T134" s="2"/>
+      <c r="U134" s="2"/>
+      <c r="V134" s="2"/>
+      <c r="W134" s="2"/>
+      <c r="X134" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y134" s="2"/>
+    </row>
+    <row r="135" spans="1:25">
+      <c r="A135" s="1">
+        <v>125</v>
+      </c>
+      <c r="B135" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C135" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="D135" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E135" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G135" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H135" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I135" s="2"/>
+      <c r="J135" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K135" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L135" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M135" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N135" s="2"/>
+      <c r="O135" s="2"/>
+      <c r="P135" s="2"/>
+      <c r="Q135" s="2"/>
+      <c r="R135" s="2"/>
+      <c r="S135" s="2"/>
+      <c r="T135" s="2"/>
+      <c r="U135" s="2"/>
+      <c r="V135" s="2"/>
+      <c r="W135" s="2"/>
+      <c r="X135" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y135" s="2"/>
+    </row>
+    <row r="136" spans="1:25">
+      <c r="A136" s="1">
+        <v>126</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="C136" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D136" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G136" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H136" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I136" s="2"/>
+      <c r="J136" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K136" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L136" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M136" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N136" s="2"/>
+      <c r="O136" s="2"/>
+      <c r="P136" s="2"/>
+      <c r="Q136" s="2"/>
+      <c r="R136" s="2"/>
+      <c r="S136" s="2"/>
+      <c r="T136" s="2"/>
+      <c r="U136" s="2"/>
+      <c r="V136" s="2"/>
+      <c r="W136" s="2"/>
+      <c r="X136" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y136" s="2"/>
+    </row>
+    <row r="137" spans="1:25">
+      <c r="A137" s="1">
+        <v>127</v>
+      </c>
+      <c r="B137" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="C137" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="D137" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E137" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G137" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H137" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I137" s="2"/>
+      <c r="J137" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K137" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L137" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="M137" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N137" s="2"/>
+      <c r="O137" s="2"/>
+      <c r="P137" s="2"/>
+      <c r="Q137" s="2"/>
+      <c r="R137" s="2"/>
+      <c r="S137" s="2"/>
+      <c r="T137" s="2"/>
+      <c r="U137" s="2"/>
+      <c r="V137" s="2"/>
+      <c r="W137" s="2"/>
+      <c r="X137" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y137" s="2"/>
+    </row>
+    <row r="138" spans="1:25">
+      <c r="A138" s="1">
+        <v>128</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H138" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I138" s="2"/>
+      <c r="J138" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="K138" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L138" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="M138" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N138" s="2"/>
+      <c r="O138" s="2"/>
+      <c r="P138" s="2"/>
+      <c r="Q138" s="2"/>
+      <c r="R138" s="2"/>
+      <c r="S138" s="2"/>
+      <c r="T138" s="2"/>
+      <c r="U138" s="2"/>
+      <c r="V138" s="2"/>
+      <c r="W138" s="2"/>
+      <c r="X138" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y138" s="2"/>
+    </row>
+    <row r="139" spans="1:25">
+      <c r="A139" s="1">
+        <v>129</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="C139" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G139" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H139" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I139" s="2"/>
+      <c r="J139" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="K139" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L139" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="M139" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N139" s="2"/>
+      <c r="O139" s="2"/>
+      <c r="P139" s="2"/>
+      <c r="Q139" s="2"/>
+      <c r="R139" s="2"/>
+      <c r="S139" s="2"/>
+      <c r="T139" s="2"/>
+      <c r="U139" s="2"/>
+      <c r="V139" s="2"/>
+      <c r="W139" s="2"/>
+      <c r="X139" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y139" s="2"/>
+    </row>
+    <row r="140" spans="1:25">
+      <c r="A140" s="1">
+        <v>130</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="D140" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E140" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H140" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I140" s="2"/>
+      <c r="J140" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="K140" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L140" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="M140" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N140" s="2"/>
+      <c r="O140" s="2"/>
+      <c r="P140" s="2"/>
+      <c r="Q140" s="2"/>
+      <c r="R140" s="2"/>
+      <c r="S140" s="2"/>
+      <c r="T140" s="2"/>
+      <c r="U140" s="2"/>
+      <c r="V140" s="2"/>
+      <c r="W140" s="2"/>
+      <c r="X140" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y140" s="2"/>
+    </row>
+    <row r="141" spans="1:25">
+      <c r="A141" s="1">
+        <v>131</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="C141" s="2" t="s">
+        <v>441</v>
+      </c>
+      <c r="D141" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E141" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F141" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G141" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H141" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I141" s="2"/>
+      <c r="J141" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="K141" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="L141" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="M141" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N141" s="2"/>
+      <c r="O141" s="2"/>
+      <c r="P141" s="2"/>
+      <c r="Q141" s="2"/>
+      <c r="R141" s="2"/>
+      <c r="S141" s="2"/>
+      <c r="T141" s="2"/>
+      <c r="U141" s="2"/>
+      <c r="V141" s="2"/>
+      <c r="W141" s="2"/>
+      <c r="X141" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y141" s="2"/>
+    </row>
+    <row r="142" spans="1:25">
+      <c r="A142" s="1">
+        <v>132</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E142" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="F142" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H142" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I142" s="2"/>
+      <c r="J142" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K142" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L142" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M142" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N142" s="2"/>
+      <c r="O142" s="2"/>
+      <c r="P142" s="2"/>
+      <c r="Q142" s="2"/>
+      <c r="R142" s="2"/>
+      <c r="S142" s="2"/>
+      <c r="T142" s="2"/>
+      <c r="U142" s="2"/>
+      <c r="V142" s="2"/>
+      <c r="W142" s="2"/>
+      <c r="X142" s="1">
+        <v>30</v>
+      </c>
+      <c r="Y142" s="2"/>
+    </row>
+    <row r="143" spans="1:25">
+      <c r="A143" s="1">
+        <v>133</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="D143" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E143" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="F143" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G143" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H143" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I143" s="2"/>
+      <c r="J143" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K143" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L143" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M143" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N143" s="2"/>
+      <c r="O143" s="2"/>
+      <c r="P143" s="2"/>
+      <c r="Q143" s="2"/>
+      <c r="R143" s="2"/>
+      <c r="S143" s="2"/>
+      <c r="T143" s="2"/>
+      <c r="U143" s="2"/>
+      <c r="V143" s="2"/>
+      <c r="W143" s="2"/>
+      <c r="X143" s="1">
+        <v>2</v>
+      </c>
+      <c r="Y143" s="2"/>
+    </row>
+    <row r="144" spans="1:25">
+      <c r="A144" s="1">
+        <v>134</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D144" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E144" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="F144" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G144" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H144" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I144" s="2"/>
+      <c r="J144" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K144" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="L144" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="M144" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N144" s="2"/>
+      <c r="O144" s="2"/>
+      <c r="P144" s="2"/>
+      <c r="Q144" s="2"/>
+      <c r="R144" s="2"/>
+      <c r="S144" s="2"/>
+      <c r="T144" s="2"/>
+      <c r="U144" s="2"/>
+      <c r="V144" s="2"/>
+      <c r="W144" s="2"/>
+      <c r="X144" s="1">
+        <v>3</v>
+      </c>
+      <c r="Y144" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>